<commit_message>
Publish VS Vitathione NAD+ skin glow guide
</commit_message>
<xml_diff>
--- a/seo-automation/sowena-seo-master-tracker.xlsx
+++ b/seo-automation/sowena-seo-master-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R648fda54eafd463d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="2" r:id="R4b2fb969a76e485a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap 100" sheetId="3" r:id="R1a203e3830af4989"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Links" sheetId="4" r:id="R54e09472e65d4b8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Notes" sheetId="5" r:id="R48723998b60749ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0d8881bafa174561"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="2" r:id="Rd99d14d59cdb4336"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap 100" sheetId="3" r:id="Rbcb635fc88b94642"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Links" sheetId="4" r:id="R7bcbc159d70c4ea1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Notes" sheetId="5" r:id="R761be5e5e7284beb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -649,7 +649,7 @@
         <x:v>Indexable URLs in updated sitemap</x:v>
       </x:c>
       <x:c r="B5" s="19" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C5" s="15"/>
       <x:c r="D5" s="20" t="str">
@@ -1327,7 +1327,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8501df8607b49d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc75f2963621c47bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1466,7 +1466,7 @@
         <x:v>SEO-002</x:v>
       </x:c>
       <x:c r="B3" s="35" t="str">
-        <x:v>VS Vitathione NAD+: professional guide for clinics and wholesale buyers</x:v>
+        <x:v>VS Vitathione NAD+: ingredients, glow goals and routine support</x:v>
       </x:c>
       <x:c r="C3" s="35" t="str">
         <x:v>NAD+ skin boosters</x:v>
@@ -1475,39 +1475,43 @@
         <x:v>Product / commercial</x:v>
       </x:c>
       <x:c r="E3" s="35" t="str">
-        <x:v>vs vitathione nad+ wholesale</x:v>
+        <x:v>vs vitathione nad ingredients</x:v>
       </x:c>
       <x:c r="F3" s="35" t="str">
         <x:v>VS Vitathione NAD+ supplier; VS Vitathione NAD+ professional guide; NAD+ aesthetic products; NAD skin booster comparison; professional skin boosters</x:v>
       </x:c>
       <x:c r="G3" s="35" t="str">
-        <x:v>Commercial investigation</x:v>
+        <x:v>Informational</x:v>
       </x:c>
       <x:c r="H3" s="35" t="str">
-        <x:v>vs-vitathione-nad-plus-professional-guide</x:v>
+        <x:v>vs-vitathione-nad-plus-skin-glow-guide</x:v>
       </x:c>
       <x:c r="I3" s="35" t="str">
-        <x:v>assets/products/vs-vitathione-nad.webp</x:v>
+        <x:v>assets/products/vs-vitathione-nad-approved.webp</x:v>
       </x:c>
       <x:c r="J3" s="35" t="str">
-        <x:v>products.html; contact.html; planned pillar: blog/what-is-nad-plus-in-professional-aesthetic-product-conversations.html</x:v>
+        <x:v>products.html; brand.html; contact.html; blog/vs-nad-plus-professional-guide.html; planned pillar: blog/what-is-nad-plus-in-professional-aesthetic-product-conversations.html</x:v>
       </x:c>
       <x:c r="K3" s="35" t="str">
-        <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
+        <x:v>https://victoriasun.net/ (official company website; dedicated official product page not available)</x:v>
       </x:c>
       <x:c r="L3" s="35" t="str">
-        <x:v>PLANNED</x:v>
-      </x:c>
-      <x:c r="M3" s="35" t="str"/>
-      <x:c r="N3" s="42"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M3" s="35" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/vs-vitathione-nad-plus-skin-glow-guide.html</x:v>
+      </x:c>
+      <x:c r="N3" s="42" t="n">
+        <x:v>46296</x:v>
+      </x:c>
       <x:c r="O3" s="35" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P3" s="42" t="n">
-        <x:v>46295</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="Q3" s="36" t="str">
-        <x:v>Keyword volume not claimed. Verify search demand, product facts, packaging, manufacturer and local regulatory context before writing.</x:v>
+        <x:v>Published with approved Sowena artwork. Ingredient names are limited to the visible packaging; no dedicated official product page was available.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1637,7 +1641,7 @@
         <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
       </x:c>
       <x:c r="J6" s="35" t="str">
-        <x:v>blog/vs-nad-plus-professional-guide.html; blog/vs-vitathione-nad-plus-professional-guide.html; blog/vs-pnad-plus-professional-guide.html; blog/vs-collagen-nad-plus-professional-guide.html; products.html</x:v>
+        <x:v>blog/vs-nad-plus-professional-guide.html; blog/vs-vitathione-nad-plus-skin-glow-guide.html; blog/vs-pnad-plus-professional-guide.html; blog/vs-collagen-nad-plus-professional-guide.html; products.html</x:v>
       </x:c>
       <x:c r="K6" s="35" t="str">
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
@@ -6332,7 +6336,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4223df69ca384793"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R372e5b39e30e4636"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6772,7 +6776,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54c21bb0eff6425f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f3c5320ec6b4148"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6916,7 +6920,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8413bf85daf54fd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a7feb9fb2e54ada"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Pause SEO schedule for batch publishing
</commit_message>
<xml_diff>
--- a/seo-automation/sowena-seo-master-tracker.xlsx
+++ b/seo-automation/sowena-seo-master-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra027a0dca38b4d4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="2" r:id="Rf55bf4ed4ad4447d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap 100" sheetId="3" r:id="R4a6b8d67bf034253"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Links" sheetId="4" r:id="R7658646a22694891"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Notes" sheetId="5" r:id="Reb05f1aa32224778"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R676978f81bd44e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="2" r:id="Ra33d45f23c644517"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap 100" sheetId="3" r:id="R92e52fc1625b43fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Links" sheetId="4" r:id="Ra17e3c9f28b44d98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Notes" sheetId="5" r:id="R2ef6a5f3f4b846c3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -984,7 +984,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="20" t="str">
-        <x:v>Publish one validated article per day at 20:00 Vietnam time. Complete SEO-003 through SEO-102 in exact order, verify product images and sources before publication, and pause automatically after the campaign reaches 100 additional live articles.</x:v>
+        <x:v>Scheduled publishing is paused. Keep SEO-004 through SEO-102 on batch hold and publish them together only after all required approved product images, sources and validations are ready and the user explicitly resumes the campaign.</x:v>
       </x:c>
     </x:row>
     <x:row r="14"/>
@@ -1840,7 +1840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red246407183c4a7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf89fc4c7ce140b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2149,12 +2149,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L5" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M5" s="56"/>
-      <x:c r="N5" s="49" t="n">
-        <x:v>46299</x:v>
-      </x:c>
+      <x:c r="N5" s="49"/>
       <x:c r="O5" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2162,7 +2160,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q5" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2200,12 +2198,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L6" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M6" s="56"/>
-      <x:c r="N6" s="49" t="n">
-        <x:v>46300</x:v>
-      </x:c>
+      <x:c r="N6" s="49"/>
       <x:c r="O6" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2213,7 +2209,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q6" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2251,12 +2247,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L7" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M7" s="56"/>
-      <x:c r="N7" s="49" t="n">
-        <x:v>46301</x:v>
-      </x:c>
+      <x:c r="N7" s="49"/>
       <x:c r="O7" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2264,7 +2258,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q7" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2302,12 +2296,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L8" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M8" s="56"/>
-      <x:c r="N8" s="49" t="n">
-        <x:v>46302</x:v>
-      </x:c>
+      <x:c r="N8" s="49"/>
       <x:c r="O8" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2315,7 +2307,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q8" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2353,12 +2345,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L9" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M9" s="56"/>
-      <x:c r="N9" s="49" t="n">
-        <x:v>46303</x:v>
-      </x:c>
+      <x:c r="N9" s="49"/>
       <x:c r="O9" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2366,7 +2356,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q9" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2404,12 +2394,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L10" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M10" s="56"/>
-      <x:c r="N10" s="49" t="n">
-        <x:v>46304</x:v>
-      </x:c>
+      <x:c r="N10" s="49"/>
       <x:c r="O10" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2417,7 +2405,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q10" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2455,12 +2443,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L11" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M11" s="56"/>
-      <x:c r="N11" s="49" t="n">
-        <x:v>46305</x:v>
-      </x:c>
+      <x:c r="N11" s="49"/>
       <x:c r="O11" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2468,7 +2454,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q11" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2506,12 +2492,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L12" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M12" s="56"/>
-      <x:c r="N12" s="49" t="n">
-        <x:v>46306</x:v>
-      </x:c>
+      <x:c r="N12" s="49"/>
       <x:c r="O12" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2519,7 +2503,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q12" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2557,12 +2541,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L13" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M13" s="56"/>
-      <x:c r="N13" s="49" t="n">
-        <x:v>46307</x:v>
-      </x:c>
+      <x:c r="N13" s="49"/>
       <x:c r="O13" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2570,7 +2552,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q13" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2608,12 +2590,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L14" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M14" s="56"/>
-      <x:c r="N14" s="49" t="n">
-        <x:v>46308</x:v>
-      </x:c>
+      <x:c r="N14" s="49"/>
       <x:c r="O14" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2621,7 +2601,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q14" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2659,12 +2639,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L15" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M15" s="56"/>
-      <x:c r="N15" s="49" t="n">
-        <x:v>46309</x:v>
-      </x:c>
+      <x:c r="N15" s="49"/>
       <x:c r="O15" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2672,7 +2650,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q15" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2710,12 +2688,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L16" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M16" s="56"/>
-      <x:c r="N16" s="49" t="n">
-        <x:v>46310</x:v>
-      </x:c>
+      <x:c r="N16" s="49"/>
       <x:c r="O16" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2723,7 +2699,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q16" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2761,12 +2737,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L17" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M17" s="56"/>
-      <x:c r="N17" s="49" t="n">
-        <x:v>46311</x:v>
-      </x:c>
+      <x:c r="N17" s="49"/>
       <x:c r="O17" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2774,7 +2748,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q17" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2812,12 +2786,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L18" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M18" s="56"/>
-      <x:c r="N18" s="49" t="n">
-        <x:v>46312</x:v>
-      </x:c>
+      <x:c r="N18" s="49"/>
       <x:c r="O18" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2825,7 +2797,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q18" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2863,12 +2835,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L19" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M19" s="56"/>
-      <x:c r="N19" s="49" t="n">
-        <x:v>46313</x:v>
-      </x:c>
+      <x:c r="N19" s="49"/>
       <x:c r="O19" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2876,7 +2846,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q19" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2914,12 +2884,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L20" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M20" s="56"/>
-      <x:c r="N20" s="49" t="n">
-        <x:v>46314</x:v>
-      </x:c>
+      <x:c r="N20" s="49"/>
       <x:c r="O20" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2927,7 +2895,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q20" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2965,12 +2933,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L21" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M21" s="56"/>
-      <x:c r="N21" s="49" t="n">
-        <x:v>46315</x:v>
-      </x:c>
+      <x:c r="N21" s="49"/>
       <x:c r="O21" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -2978,7 +2944,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q21" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -3016,12 +2982,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L22" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M22" s="56"/>
-      <x:c r="N22" s="49" t="n">
-        <x:v>46316</x:v>
-      </x:c>
+      <x:c r="N22" s="49"/>
       <x:c r="O22" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3029,7 +2993,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q22" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -3067,12 +3031,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L23" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M23" s="56"/>
-      <x:c r="N23" s="49" t="n">
-        <x:v>46317</x:v>
-      </x:c>
+      <x:c r="N23" s="49"/>
       <x:c r="O23" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3080,7 +3042,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q23" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -3118,12 +3080,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L24" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M24" s="56"/>
-      <x:c r="N24" s="49" t="n">
-        <x:v>46318</x:v>
-      </x:c>
+      <x:c r="N24" s="49"/>
       <x:c r="O24" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3131,7 +3091,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q24" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -3169,12 +3129,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L25" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M25" s="56"/>
-      <x:c r="N25" s="49" t="n">
-        <x:v>46319</x:v>
-      </x:c>
+      <x:c r="N25" s="49"/>
       <x:c r="O25" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3182,7 +3140,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q25" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -3220,12 +3178,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L26" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M26" s="56"/>
-      <x:c r="N26" s="49" t="n">
-        <x:v>46320</x:v>
-      </x:c>
+      <x:c r="N26" s="49"/>
       <x:c r="O26" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3233,7 +3189,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q26" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -3271,12 +3227,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L27" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M27" s="56"/>
-      <x:c r="N27" s="49" t="n">
-        <x:v>46321</x:v>
-      </x:c>
+      <x:c r="N27" s="49"/>
       <x:c r="O27" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3284,7 +3238,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q27" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -3322,12 +3276,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L28" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M28" s="56"/>
-      <x:c r="N28" s="49" t="n">
-        <x:v>46322</x:v>
-      </x:c>
+      <x:c r="N28" s="49"/>
       <x:c r="O28" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3335,7 +3287,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q28" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -3373,12 +3325,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L29" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M29" s="56"/>
-      <x:c r="N29" s="49" t="n">
-        <x:v>46323</x:v>
-      </x:c>
+      <x:c r="N29" s="49"/>
       <x:c r="O29" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3386,7 +3336,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q29" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -3424,12 +3374,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L30" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M30" s="56"/>
-      <x:c r="N30" s="49" t="n">
-        <x:v>46324</x:v>
-      </x:c>
+      <x:c r="N30" s="49"/>
       <x:c r="O30" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3437,7 +3385,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q30" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -3475,12 +3423,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L31" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M31" s="56"/>
-      <x:c r="N31" s="49" t="n">
-        <x:v>46325</x:v>
-      </x:c>
+      <x:c r="N31" s="49"/>
       <x:c r="O31" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3488,7 +3434,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q31" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -3526,12 +3472,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L32" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M32" s="56"/>
-      <x:c r="N32" s="49" t="n">
-        <x:v>46326</x:v>
-      </x:c>
+      <x:c r="N32" s="49"/>
       <x:c r="O32" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3539,7 +3483,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q32" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -3577,12 +3521,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L33" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M33" s="56"/>
-      <x:c r="N33" s="49" t="n">
-        <x:v>46327</x:v>
-      </x:c>
+      <x:c r="N33" s="49"/>
       <x:c r="O33" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3590,7 +3532,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q33" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -3628,12 +3570,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L34" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M34" s="56"/>
-      <x:c r="N34" s="49" t="n">
-        <x:v>46328</x:v>
-      </x:c>
+      <x:c r="N34" s="49"/>
       <x:c r="O34" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3641,7 +3581,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q34" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -3679,12 +3619,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L35" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M35" s="56"/>
-      <x:c r="N35" s="49" t="n">
-        <x:v>46329</x:v>
-      </x:c>
+      <x:c r="N35" s="49"/>
       <x:c r="O35" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3692,7 +3630,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q35" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -3730,12 +3668,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L36" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M36" s="56"/>
-      <x:c r="N36" s="49" t="n">
-        <x:v>46330</x:v>
-      </x:c>
+      <x:c r="N36" s="49"/>
       <x:c r="O36" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3743,7 +3679,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q36" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -3781,12 +3717,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L37" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M37" s="56"/>
-      <x:c r="N37" s="49" t="n">
-        <x:v>46331</x:v>
-      </x:c>
+      <x:c r="N37" s="49"/>
       <x:c r="O37" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3794,7 +3728,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q37" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -3832,12 +3766,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L38" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M38" s="56"/>
-      <x:c r="N38" s="49" t="n">
-        <x:v>46332</x:v>
-      </x:c>
+      <x:c r="N38" s="49"/>
       <x:c r="O38" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3845,7 +3777,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q38" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -3883,12 +3815,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L39" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M39" s="56"/>
-      <x:c r="N39" s="49" t="n">
-        <x:v>46333</x:v>
-      </x:c>
+      <x:c r="N39" s="49"/>
       <x:c r="O39" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3896,7 +3826,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q39" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -3934,12 +3864,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L40" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M40" s="56"/>
-      <x:c r="N40" s="49" t="n">
-        <x:v>46334</x:v>
-      </x:c>
+      <x:c r="N40" s="49"/>
       <x:c r="O40" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3947,7 +3875,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q40" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -3985,12 +3913,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L41" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M41" s="56"/>
-      <x:c r="N41" s="49" t="n">
-        <x:v>46335</x:v>
-      </x:c>
+      <x:c r="N41" s="49"/>
       <x:c r="O41" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -3998,7 +3924,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q41" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -4036,12 +3962,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L42" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M42" s="56"/>
-      <x:c r="N42" s="49" t="n">
-        <x:v>46336</x:v>
-      </x:c>
+      <x:c r="N42" s="49"/>
       <x:c r="O42" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4049,7 +3973,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q42" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -4087,12 +4011,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L43" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M43" s="56"/>
-      <x:c r="N43" s="49" t="n">
-        <x:v>46337</x:v>
-      </x:c>
+      <x:c r="N43" s="49"/>
       <x:c r="O43" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4100,7 +4022,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q43" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -4138,12 +4060,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L44" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M44" s="56"/>
-      <x:c r="N44" s="49" t="n">
-        <x:v>46338</x:v>
-      </x:c>
+      <x:c r="N44" s="49"/>
       <x:c r="O44" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4151,7 +4071,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q44" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -4189,12 +4109,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L45" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M45" s="56"/>
-      <x:c r="N45" s="49" t="n">
-        <x:v>46339</x:v>
-      </x:c>
+      <x:c r="N45" s="49"/>
       <x:c r="O45" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4202,7 +4120,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q45" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -4240,12 +4158,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L46" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M46" s="56"/>
-      <x:c r="N46" s="49" t="n">
-        <x:v>46340</x:v>
-      </x:c>
+      <x:c r="N46" s="49"/>
       <x:c r="O46" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4253,7 +4169,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q46" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -4291,12 +4207,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L47" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M47" s="56"/>
-      <x:c r="N47" s="49" t="n">
-        <x:v>46341</x:v>
-      </x:c>
+      <x:c r="N47" s="49"/>
       <x:c r="O47" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4304,7 +4218,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q47" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -4342,12 +4256,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L48" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M48" s="56"/>
-      <x:c r="N48" s="49" t="n">
-        <x:v>46342</x:v>
-      </x:c>
+      <x:c r="N48" s="49"/>
       <x:c r="O48" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4355,7 +4267,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q48" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -4393,12 +4305,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L49" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M49" s="56"/>
-      <x:c r="N49" s="49" t="n">
-        <x:v>46343</x:v>
-      </x:c>
+      <x:c r="N49" s="49"/>
       <x:c r="O49" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4406,7 +4316,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q49" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -4444,12 +4354,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L50" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M50" s="56"/>
-      <x:c r="N50" s="49" t="n">
-        <x:v>46344</x:v>
-      </x:c>
+      <x:c r="N50" s="49"/>
       <x:c r="O50" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4457,7 +4365,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q50" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -4495,12 +4403,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L51" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M51" s="56"/>
-      <x:c r="N51" s="49" t="n">
-        <x:v>46345</x:v>
-      </x:c>
+      <x:c r="N51" s="49"/>
       <x:c r="O51" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4508,7 +4414,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q51" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -4546,12 +4452,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L52" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M52" s="56"/>
-      <x:c r="N52" s="49" t="n">
-        <x:v>46346</x:v>
-      </x:c>
+      <x:c r="N52" s="49"/>
       <x:c r="O52" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4559,7 +4463,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q52" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -4597,12 +4501,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L53" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M53" s="56"/>
-      <x:c r="N53" s="49" t="n">
-        <x:v>46347</x:v>
-      </x:c>
+      <x:c r="N53" s="49"/>
       <x:c r="O53" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4610,7 +4512,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q53" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -4648,12 +4550,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L54" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M54" s="56"/>
-      <x:c r="N54" s="49" t="n">
-        <x:v>46348</x:v>
-      </x:c>
+      <x:c r="N54" s="49"/>
       <x:c r="O54" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4661,7 +4561,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q54" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -4699,12 +4599,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L55" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M55" s="56"/>
-      <x:c r="N55" s="49" t="n">
-        <x:v>46349</x:v>
-      </x:c>
+      <x:c r="N55" s="49"/>
       <x:c r="O55" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4712,7 +4610,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q55" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -4750,12 +4648,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L56" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M56" s="56"/>
-      <x:c r="N56" s="49" t="n">
-        <x:v>46350</x:v>
-      </x:c>
+      <x:c r="N56" s="49"/>
       <x:c r="O56" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4763,7 +4659,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q56" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -4801,12 +4697,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L57" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M57" s="56"/>
-      <x:c r="N57" s="49" t="n">
-        <x:v>46351</x:v>
-      </x:c>
+      <x:c r="N57" s="49"/>
       <x:c r="O57" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4814,7 +4708,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q57" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -4852,12 +4746,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L58" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M58" s="56"/>
-      <x:c r="N58" s="49" t="n">
-        <x:v>46352</x:v>
-      </x:c>
+      <x:c r="N58" s="49"/>
       <x:c r="O58" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4865,7 +4757,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q58" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -4903,12 +4795,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L59" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M59" s="56"/>
-      <x:c r="N59" s="49" t="n">
-        <x:v>46353</x:v>
-      </x:c>
+      <x:c r="N59" s="49"/>
       <x:c r="O59" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4916,7 +4806,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q59" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -4954,12 +4844,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L60" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M60" s="56"/>
-      <x:c r="N60" s="49" t="n">
-        <x:v>46354</x:v>
-      </x:c>
+      <x:c r="N60" s="49"/>
       <x:c r="O60" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -4967,7 +4855,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q60" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -5005,12 +4893,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L61" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M61" s="56"/>
-      <x:c r="N61" s="49" t="n">
-        <x:v>46355</x:v>
-      </x:c>
+      <x:c r="N61" s="49"/>
       <x:c r="O61" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5018,7 +4904,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q61" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -5056,12 +4942,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L62" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M62" s="56"/>
-      <x:c r="N62" s="49" t="n">
-        <x:v>46356</x:v>
-      </x:c>
+      <x:c r="N62" s="49"/>
       <x:c r="O62" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5069,7 +4953,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q62" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -5107,12 +4991,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L63" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M63" s="56"/>
-      <x:c r="N63" s="49" t="n">
-        <x:v>46357</x:v>
-      </x:c>
+      <x:c r="N63" s="49"/>
       <x:c r="O63" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5120,7 +5002,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q63" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -5158,12 +5040,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L64" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M64" s="56"/>
-      <x:c r="N64" s="49" t="n">
-        <x:v>46358</x:v>
-      </x:c>
+      <x:c r="N64" s="49"/>
       <x:c r="O64" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5171,7 +5051,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q64" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -5209,12 +5089,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L65" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M65" s="56"/>
-      <x:c r="N65" s="49" t="n">
-        <x:v>46359</x:v>
-      </x:c>
+      <x:c r="N65" s="49"/>
       <x:c r="O65" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5222,7 +5100,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q65" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -5260,12 +5138,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L66" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M66" s="56"/>
-      <x:c r="N66" s="49" t="n">
-        <x:v>46360</x:v>
-      </x:c>
+      <x:c r="N66" s="49"/>
       <x:c r="O66" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5273,7 +5149,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q66" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -5311,12 +5187,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L67" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M67" s="56"/>
-      <x:c r="N67" s="49" t="n">
-        <x:v>46361</x:v>
-      </x:c>
+      <x:c r="N67" s="49"/>
       <x:c r="O67" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5324,7 +5198,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q67" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -5362,12 +5236,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L68" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M68" s="56"/>
-      <x:c r="N68" s="49" t="n">
-        <x:v>46362</x:v>
-      </x:c>
+      <x:c r="N68" s="49"/>
       <x:c r="O68" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5375,7 +5247,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q68" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -5413,12 +5285,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L69" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M69" s="56"/>
-      <x:c r="N69" s="49" t="n">
-        <x:v>46363</x:v>
-      </x:c>
+      <x:c r="N69" s="49"/>
       <x:c r="O69" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5426,7 +5296,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q69" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -5464,12 +5334,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L70" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M70" s="56"/>
-      <x:c r="N70" s="49" t="n">
-        <x:v>46364</x:v>
-      </x:c>
+      <x:c r="N70" s="49"/>
       <x:c r="O70" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5477,7 +5345,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q70" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -5515,12 +5383,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L71" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M71" s="56"/>
-      <x:c r="N71" s="49" t="n">
-        <x:v>46365</x:v>
-      </x:c>
+      <x:c r="N71" s="49"/>
       <x:c r="O71" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5528,7 +5394,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q71" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -5566,12 +5432,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L72" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M72" s="56"/>
-      <x:c r="N72" s="49" t="n">
-        <x:v>46366</x:v>
-      </x:c>
+      <x:c r="N72" s="49"/>
       <x:c r="O72" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5579,7 +5443,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q72" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -5617,12 +5481,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L73" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M73" s="56"/>
-      <x:c r="N73" s="49" t="n">
-        <x:v>46367</x:v>
-      </x:c>
+      <x:c r="N73" s="49"/>
       <x:c r="O73" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5630,7 +5492,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q73" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -5668,12 +5530,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L74" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M74" s="56"/>
-      <x:c r="N74" s="49" t="n">
-        <x:v>46368</x:v>
-      </x:c>
+      <x:c r="N74" s="49"/>
       <x:c r="O74" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5681,7 +5541,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q74" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -5719,12 +5579,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L75" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M75" s="56"/>
-      <x:c r="N75" s="49" t="n">
-        <x:v>46369</x:v>
-      </x:c>
+      <x:c r="N75" s="49"/>
       <x:c r="O75" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5732,7 +5590,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q75" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -5770,12 +5628,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L76" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M76" s="56"/>
-      <x:c r="N76" s="49" t="n">
-        <x:v>46370</x:v>
-      </x:c>
+      <x:c r="N76" s="49"/>
       <x:c r="O76" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5783,7 +5639,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q76" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -5821,12 +5677,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L77" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M77" s="56"/>
-      <x:c r="N77" s="49" t="n">
-        <x:v>46371</x:v>
-      </x:c>
+      <x:c r="N77" s="49"/>
       <x:c r="O77" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5834,7 +5688,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q77" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -5872,12 +5726,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L78" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M78" s="56"/>
-      <x:c r="N78" s="49" t="n">
-        <x:v>46372</x:v>
-      </x:c>
+      <x:c r="N78" s="49"/>
       <x:c r="O78" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5885,7 +5737,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q78" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -5923,12 +5775,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L79" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M79" s="56"/>
-      <x:c r="N79" s="49" t="n">
-        <x:v>46373</x:v>
-      </x:c>
+      <x:c r="N79" s="49"/>
       <x:c r="O79" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5936,7 +5786,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q79" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -5974,12 +5824,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L80" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M80" s="56"/>
-      <x:c r="N80" s="49" t="n">
-        <x:v>46374</x:v>
-      </x:c>
+      <x:c r="N80" s="49"/>
       <x:c r="O80" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -5987,7 +5835,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q80" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -6025,12 +5873,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L81" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M81" s="56"/>
-      <x:c r="N81" s="49" t="n">
-        <x:v>46375</x:v>
-      </x:c>
+      <x:c r="N81" s="49"/>
       <x:c r="O81" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6038,7 +5884,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q81" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -6076,12 +5922,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L82" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M82" s="56"/>
-      <x:c r="N82" s="49" t="n">
-        <x:v>46376</x:v>
-      </x:c>
+      <x:c r="N82" s="49"/>
       <x:c r="O82" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6089,7 +5933,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q82" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -6127,12 +5971,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L83" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M83" s="56"/>
-      <x:c r="N83" s="49" t="n">
-        <x:v>46377</x:v>
-      </x:c>
+      <x:c r="N83" s="49"/>
       <x:c r="O83" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6140,7 +5982,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q83" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -6178,12 +6020,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L84" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M84" s="56"/>
-      <x:c r="N84" s="49" t="n">
-        <x:v>46378</x:v>
-      </x:c>
+      <x:c r="N84" s="49"/>
       <x:c r="O84" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6191,7 +6031,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q84" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -6229,12 +6069,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L85" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M85" s="56"/>
-      <x:c r="N85" s="49" t="n">
-        <x:v>46379</x:v>
-      </x:c>
+      <x:c r="N85" s="49"/>
       <x:c r="O85" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6242,7 +6080,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q85" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -6280,12 +6118,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L86" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M86" s="56"/>
-      <x:c r="N86" s="49" t="n">
-        <x:v>46380</x:v>
-      </x:c>
+      <x:c r="N86" s="49"/>
       <x:c r="O86" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6293,7 +6129,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q86" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -6331,12 +6167,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L87" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M87" s="56"/>
-      <x:c r="N87" s="49" t="n">
-        <x:v>46381</x:v>
-      </x:c>
+      <x:c r="N87" s="49"/>
       <x:c r="O87" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6344,7 +6178,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q87" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -6382,12 +6216,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L88" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M88" s="56"/>
-      <x:c r="N88" s="49" t="n">
-        <x:v>46382</x:v>
-      </x:c>
+      <x:c r="N88" s="49"/>
       <x:c r="O88" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6395,7 +6227,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q88" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -6433,12 +6265,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L89" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M89" s="56"/>
-      <x:c r="N89" s="49" t="n">
-        <x:v>46383</x:v>
-      </x:c>
+      <x:c r="N89" s="49"/>
       <x:c r="O89" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6446,7 +6276,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q89" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -6484,12 +6314,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L90" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M90" s="56"/>
-      <x:c r="N90" s="49" t="n">
-        <x:v>46384</x:v>
-      </x:c>
+      <x:c r="N90" s="49"/>
       <x:c r="O90" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6497,7 +6325,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q90" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -6535,12 +6363,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L91" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M91" s="56"/>
-      <x:c r="N91" s="49" t="n">
-        <x:v>46385</x:v>
-      </x:c>
+      <x:c r="N91" s="49"/>
       <x:c r="O91" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6548,7 +6374,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q91" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -6586,12 +6412,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L92" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M92" s="56"/>
-      <x:c r="N92" s="49" t="n">
-        <x:v>46386</x:v>
-      </x:c>
+      <x:c r="N92" s="49"/>
       <x:c r="O92" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6599,7 +6423,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q92" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -6637,12 +6461,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L93" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M93" s="56"/>
-      <x:c r="N93" s="49" t="n">
-        <x:v>46387</x:v>
-      </x:c>
+      <x:c r="N93" s="49"/>
       <x:c r="O93" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6650,7 +6472,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q93" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -6688,12 +6510,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L94" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M94" s="56"/>
-      <x:c r="N94" s="49" t="n">
-        <x:v>46388</x:v>
-      </x:c>
+      <x:c r="N94" s="49"/>
       <x:c r="O94" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6701,7 +6521,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q94" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -6739,12 +6559,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L95" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M95" s="56"/>
-      <x:c r="N95" s="49" t="n">
-        <x:v>46389</x:v>
-      </x:c>
+      <x:c r="N95" s="49"/>
       <x:c r="O95" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6752,7 +6570,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q95" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -6790,12 +6608,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L96" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M96" s="56"/>
-      <x:c r="N96" s="49" t="n">
-        <x:v>46390</x:v>
-      </x:c>
+      <x:c r="N96" s="49"/>
       <x:c r="O96" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6803,7 +6619,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q96" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -6841,12 +6657,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L97" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M97" s="56"/>
-      <x:c r="N97" s="49" t="n">
-        <x:v>46391</x:v>
-      </x:c>
+      <x:c r="N97" s="49"/>
       <x:c r="O97" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6854,7 +6668,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q97" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -6892,12 +6706,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L98" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M98" s="56"/>
-      <x:c r="N98" s="49" t="n">
-        <x:v>46392</x:v>
-      </x:c>
+      <x:c r="N98" s="49"/>
       <x:c r="O98" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6905,7 +6717,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q98" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -6943,12 +6755,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L99" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M99" s="56"/>
-      <x:c r="N99" s="49" t="n">
-        <x:v>46393</x:v>
-      </x:c>
+      <x:c r="N99" s="49"/>
       <x:c r="O99" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -6956,7 +6766,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q99" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -6994,12 +6804,10 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L100" s="56" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M100" s="56"/>
-      <x:c r="N100" s="49" t="n">
-        <x:v>46394</x:v>
-      </x:c>
+      <x:c r="N100" s="49"/>
       <x:c r="O100" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -7007,7 +6815,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q100" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -7045,12 +6853,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L101" s="59" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M101" s="59"/>
-      <x:c r="N101" s="50" t="n">
-        <x:v>46395</x:v>
-      </x:c>
+      <x:c r="N101" s="50"/>
       <x:c r="O101" s="59" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -7058,7 +6864,7 @@
         <x:v>46295</x:v>
       </x:c>
       <x:c r="Q101" s="60" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA.</x:v>
+        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -7096,12 +6902,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L102" s="61" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M102" s="61"/>
-      <x:c r="N102" s="62" t="n">
-        <x:v>46396</x:v>
-      </x:c>
+      <x:c r="N102" s="62"/>
       <x:c r="O102" s="61" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -7109,7 +6913,7 @@
         <x:v>46298</x:v>
       </x:c>
       <x:c r="Q102" s="61" t="str">
-        <x:v>Distinct content-gap article comparing daily topical care with professional product categories. Educational value first; no procedure instructions.</x:v>
+        <x:v>Distinct content-gap article comparing daily topical care with professional product categories. Educational value first; no procedure instructions. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -7147,12 +6951,10 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L103" s="61" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>BATCH HOLD</x:v>
       </x:c>
       <x:c r="M103" s="61"/>
-      <x:c r="N103" s="62" t="n">
-        <x:v>46397</x:v>
-      </x:c>
+      <x:c r="N103" s="62"/>
       <x:c r="O103" s="61" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
@@ -7160,7 +6962,7 @@
         <x:v>46298</x:v>
       </x:c>
       <x:c r="Q103" s="61" t="str">
-        <x:v>Distinct content-gap article for readers with reactive or barrier-stressed skin. Avoid diagnosis and recommend qualified consultation.</x:v>
+        <x:v>Distinct content-gap article for readers with reactive or barrier-stressed skin. Avoid diagnosis and recommend qualified consultation. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7183,7 +6985,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R176b18adb1874236"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re195fc59678a4741"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7835,7 +7637,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9608665af042e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79ad121cef434411"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8051,7 +7853,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec58942517b2496b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0136d7777f0b4e83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record verified SEO batch publication
</commit_message>
<xml_diff>
--- a/seo-automation/sowena-seo-master-tracker.xlsx
+++ b/seo-automation/sowena-seo-master-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R676978f81bd44e9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="2" r:id="Ra33d45f23c644517"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap 100" sheetId="3" r:id="R92e52fc1625b43fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Links" sheetId="4" r:id="Ra17e3c9f28b44d98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Notes" sheetId="5" r:id="R2ef6a5f3f4b846c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R699c1091a7bf4415"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="2" r:id="Ra25c7075a89c4c66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap 100" sheetId="3" r:id="Ra81c42edcfe54bec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Links" sheetId="4" r:id="R1eb16988072b45b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Notes" sheetId="5" r:id="Raa454c8245364d4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -984,7 +984,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="20" t="str">
-        <x:v>Scheduled publishing is paused. Keep SEO-004 through SEO-102 on batch hold and publish them together only after all required approved product images, sources and validations are ready and the user explicitly resumes the campaign.</x:v>
+        <x:v>Campaign status: 63 of 100 additional articles are live. The remaining 37 product articles are on hold until approved product images are added. Daily publishing automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="14"/>
@@ -1840,7 +1840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf89fc4c7ce140b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4711cb6e0fe6450d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2140,7 +2140,7 @@
         <x:v>vs-collagen-nad-plus-professional-guide</x:v>
       </x:c>
       <x:c r="I5" s="56" t="str">
-        <x:v>assets/products/vs-collagen-nad.webp</x:v>
+        <x:v>assets/products/vs-collagen-nad-plus-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J5" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/what-is-nad-plus-in-professional-aesthetic-product-conversations.html</x:v>
@@ -2149,18 +2149,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L5" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M5" s="56"/>
-      <x:c r="N5" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M5" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/vs-collagen-nad-plus-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N5" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O5" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P5" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q5" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2189,7 +2193,7 @@
         <x:v>what-is-nad-plus-in-professional-aesthetic-product-conversations</x:v>
       </x:c>
       <x:c r="I6" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/what-is-nad-plus-in-professional-aesthetic-product-conversations.webp</x:v>
       </x:c>
       <x:c r="J6" s="56" t="str">
         <x:v>blog/vs-nad-plus-professional-guide.html; blog/vs-vitathione-nad-plus-skin-glow-guide.html; blog/vs-pnad-plus-professional-guide.html; blog/vs-collagen-nad-plus-professional-guide.html; products.html</x:v>
@@ -2198,18 +2202,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L6" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M6" s="56"/>
-      <x:c r="N6" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M6" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/what-is-nad-plus-in-professional-aesthetic-product-conversations.html</x:v>
+      </x:c>
+      <x:c r="N6" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O6" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P6" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q6" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2238,7 +2246,7 @@
         <x:v>vs-multi-lamellar-nad-plus-professional-guide</x:v>
       </x:c>
       <x:c r="I7" s="56" t="str">
-        <x:v>assets/products/vs-multi-lamellar-nad.webp</x:v>
+        <x:v>assets/products/vs-multi-lamellar-nad-plus-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J7" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-compare-nad-plus-skin-booster-categories-without-overstating-claims.html</x:v>
@@ -2247,18 +2255,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L7" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M7" s="56"/>
-      <x:c r="N7" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M7" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/vs-multi-lamellar-nad-plus-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N7" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O7" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P7" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q7" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2287,7 +2299,7 @@
         <x:v>vs-toxnad-nad-plus-professional-guide</x:v>
       </x:c>
       <x:c r="I8" s="56" t="str">
-        <x:v>assets/products/vs-toxnad-nad.webp</x:v>
+        <x:v>assets/products/vs-toxnad-nad-plus-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J8" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-compare-nad-plus-skin-booster-categories-without-overstating-claims.html</x:v>
@@ -2296,18 +2308,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L8" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M8" s="56"/>
-      <x:c r="N8" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M8" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/vs-toxnad-nad-plus-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N8" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O8" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P8" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q8" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2336,7 +2352,7 @@
         <x:v>nad-plus-complex-professional-guide</x:v>
       </x:c>
       <x:c r="I9" s="56" t="str">
-        <x:v>assets/products/nad-complex.webp</x:v>
+        <x:v>assets/products/nad-plus-complex-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J9" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-compare-nad-plus-skin-booster-categories-without-overstating-claims.html</x:v>
@@ -2345,18 +2361,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L9" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M9" s="56"/>
-      <x:c r="N9" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M9" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/nad-plus-complex-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N9" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O9" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P9" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q9" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2385,7 +2405,7 @@
         <x:v>nadigo-plus-professional-guide</x:v>
       </x:c>
       <x:c r="I10" s="56" t="str">
-        <x:v>assets/products/nadigo.webp</x:v>
+        <x:v>assets/products/nadigo-plus-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J10" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-compare-nad-plus-skin-booster-categories-without-overstating-claims.html</x:v>
@@ -2394,18 +2414,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L10" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M10" s="56"/>
-      <x:c r="N10" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M10" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/nadigo-plus-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N10" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O10" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P10" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q10" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2434,7 +2458,7 @@
         <x:v>how-to-compare-nad-plus-skin-booster-categories-without-overstating-claims</x:v>
       </x:c>
       <x:c r="I11" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/how-to-compare-nad-plus-skin-booster-categories-without-overstating-claims.webp</x:v>
       </x:c>
       <x:c r="J11" s="56" t="str">
         <x:v>blog/vs-multi-lamellar-nad-plus-professional-guide.html; blog/vs-toxnad-nad-plus-professional-guide.html; blog/nad-plus-complex-professional-guide.html; blog/nadigo-plus-professional-guide.html; products.html</x:v>
@@ -2443,18 +2467,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L11" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M11" s="56"/>
-      <x:c r="N11" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M11" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/how-to-compare-nad-plus-skin-booster-categories-without-overstating-claims.html</x:v>
+      </x:c>
+      <x:c r="N11" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O11" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P11" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q11" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2483,7 +2511,7 @@
         <x:v>puri-pdrn-professional-guide</x:v>
       </x:c>
       <x:c r="I12" s="56" t="str">
-        <x:v>assets/products/puri-pdrn.webp</x:v>
+        <x:v>assets/products/puri-pdrn-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J12" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/pdrn-vs-pn-skin-boosters-terminology-evidence-and-buyer-questions.html</x:v>
@@ -2492,18 +2520,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L12" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M12" s="56"/>
-      <x:c r="N12" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M12" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/puri-pdrn-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N12" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O12" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P12" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q12" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2532,7 +2564,7 @@
         <x:v>reglory-pn-plus-professional-guide</x:v>
       </x:c>
       <x:c r="I13" s="56" t="str">
-        <x:v>assets/products/reglory-pn-plus.webp</x:v>
+        <x:v>assets/products/reglory-pn-plus-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J13" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/pdrn-vs-pn-skin-boosters-terminology-evidence-and-buyer-questions.html</x:v>
@@ -2541,18 +2573,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L13" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M13" s="56"/>
-      <x:c r="N13" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M13" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/reglory-pn-plus-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N13" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O13" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P13" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q13" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2581,7 +2617,7 @@
         <x:v>aqua-pn-professional-guide</x:v>
       </x:c>
       <x:c r="I14" s="56" t="str">
-        <x:v>assets/products/aqua-pn.webp</x:v>
+        <x:v>assets/products/aqua-pn-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J14" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/pdrn-vs-pn-skin-boosters-terminology-evidence-and-buyer-questions.html</x:v>
@@ -2590,18 +2626,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L14" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M14" s="56"/>
-      <x:c r="N14" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M14" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/aqua-pn-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N14" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O14" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P14" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q14" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2630,7 +2670,7 @@
         <x:v>kiara-reju-professional-guide</x:v>
       </x:c>
       <x:c r="I15" s="56" t="str">
-        <x:v>assets/products/kiara-reju.webp</x:v>
+        <x:v>assets/products/kiara-reju-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J15" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/pdrn-vs-pn-skin-boosters-terminology-evidence-and-buyer-questions.html</x:v>
@@ -2639,18 +2679,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L15" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M15" s="56"/>
-      <x:c r="N15" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M15" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/kiara-reju-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N15" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O15" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P15" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q15" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2679,7 +2723,7 @@
         <x:v>pdrn-vs-pn-skin-boosters-terminology-evidence-and-buyer-questions</x:v>
       </x:c>
       <x:c r="I16" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/pdrn-vs-pn-skin-boosters-terminology-evidence-and-buyer-questions.webp</x:v>
       </x:c>
       <x:c r="J16" s="56" t="str">
         <x:v>blog/puri-pdrn-professional-guide.html; blog/reglory-pn-plus-professional-guide.html; blog/aqua-pn-professional-guide.html; blog/kiara-reju-professional-guide.html; products.html</x:v>
@@ -2688,18 +2732,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L16" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M16" s="56"/>
-      <x:c r="N16" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M16" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/pdrn-vs-pn-skin-boosters-terminology-evidence-and-buyer-questions.html</x:v>
+      </x:c>
+      <x:c r="N16" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O16" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P16" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q16" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2728,7 +2776,7 @@
         <x:v>rejuran-healer-new-professional-guide</x:v>
       </x:c>
       <x:c r="I17" s="56" t="str">
-        <x:v>assets/products/rejuran-healer-new.webp</x:v>
+        <x:v>assets/products/rejuran-healer-new-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J17" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/rejuran-product-range-explained-for-professional-buyers.html</x:v>
@@ -2737,18 +2785,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L17" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M17" s="56"/>
-      <x:c r="N17" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M17" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/rejuran-healer-new-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N17" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O17" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P17" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q17" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2777,7 +2829,7 @@
         <x:v>rejuran-i-new-professional-guide</x:v>
       </x:c>
       <x:c r="I18" s="56" t="str">
-        <x:v>assets/products/rejuran-i-new.webp</x:v>
+        <x:v>assets/products/rejuran-i-new-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J18" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/rejuran-product-range-explained-for-professional-buyers.html</x:v>
@@ -2786,18 +2838,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L18" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M18" s="56"/>
-      <x:c r="N18" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M18" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/rejuran-i-new-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N18" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O18" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P18" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q18" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2826,7 +2882,7 @@
         <x:v>rejuran-s-new-professional-guide</x:v>
       </x:c>
       <x:c r="I19" s="56" t="str">
-        <x:v>assets/products/rejuran-s-new.webp</x:v>
+        <x:v>assets/products/rejuran-s-new-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J19" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/rejuran-product-range-explained-for-professional-buyers.html</x:v>
@@ -2835,18 +2891,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L19" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M19" s="56"/>
-      <x:c r="N19" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M19" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/rejuran-s-new-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N19" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O19" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P19" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q19" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2875,7 +2935,7 @@
         <x:v>rejuran-hb-new-professional-guide</x:v>
       </x:c>
       <x:c r="I20" s="56" t="str">
-        <x:v>assets/products/rejuran-hb-new.webp</x:v>
+        <x:v>assets/products/rejuran-hb-new-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J20" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/rejuran-product-range-explained-for-professional-buyers.html</x:v>
@@ -2884,18 +2944,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L20" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M20" s="56"/>
-      <x:c r="N20" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M20" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/rejuran-hb-new-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N20" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O20" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P20" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q20" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -2924,7 +2988,7 @@
         <x:v>rejuran-product-range-explained-for-professional-buyers</x:v>
       </x:c>
       <x:c r="I21" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/rejuran-product-range-explained-for-professional-buyers.webp</x:v>
       </x:c>
       <x:c r="J21" s="56" t="str">
         <x:v>blog/rejuran-healer-new-professional-guide.html; blog/rejuran-i-new-professional-guide.html; blog/rejuran-s-new-professional-guide.html; blog/rejuran-hb-new-professional-guide.html; products.html</x:v>
@@ -2933,18 +2997,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L21" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M21" s="56"/>
-      <x:c r="N21" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M21" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/rejuran-product-range-explained-for-professional-buyers.html</x:v>
+      </x:c>
+      <x:c r="N21" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O21" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P21" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q21" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -2973,7 +3041,7 @@
         <x:v>vitaran-hp-professional-guide</x:v>
       </x:c>
       <x:c r="I22" s="56" t="str">
-        <x:v>assets/products/vitaran-hp.webp</x:v>
+        <x:v>assets/products/vitaran-hp-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J22" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-professional-buyers-compare-polynucleotide-product-categories.html</x:v>
@@ -2982,18 +3050,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L22" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M22" s="56"/>
-      <x:c r="N22" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M22" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/vitaran-hp-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N22" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O22" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P22" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q22" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -3022,7 +3094,7 @@
         <x:v>vitaran-i-professional-guide</x:v>
       </x:c>
       <x:c r="I23" s="56" t="str">
-        <x:v>assets/products/vitaran-i.webp</x:v>
+        <x:v>assets/products/vitaran-i-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J23" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-professional-buyers-compare-polynucleotide-product-categories.html</x:v>
@@ -3031,18 +3103,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L23" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M23" s="56"/>
-      <x:c r="N23" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M23" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/vitaran-i-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N23" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O23" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P23" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q23" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -3071,7 +3147,7 @@
         <x:v>vitaran-s-professional-guide</x:v>
       </x:c>
       <x:c r="I24" s="56" t="str">
-        <x:v>assets/products/vitaran-s.webp</x:v>
+        <x:v>assets/products/vitaran-s-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J24" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-professional-buyers-compare-polynucleotide-product-categories.html</x:v>
@@ -3080,18 +3156,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L24" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M24" s="56"/>
-      <x:c r="N24" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M24" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/vitaran-s-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N24" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O24" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P24" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q24" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -3120,7 +3200,7 @@
         <x:v>placentex-professional-guide</x:v>
       </x:c>
       <x:c r="I25" s="56" t="str">
-        <x:v>assets/products/placentex.webp</x:v>
+        <x:v>assets/products/placentex-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J25" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-professional-buyers-compare-polynucleotide-product-categories.html</x:v>
@@ -3129,18 +3209,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L25" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M25" s="56"/>
-      <x:c r="N25" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M25" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/placentex-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N25" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O25" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P25" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q25" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -3169,7 +3253,7 @@
         <x:v>how-professional-buyers-compare-polynucleotide-product-categories</x:v>
       </x:c>
       <x:c r="I26" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/how-professional-buyers-compare-polynucleotide-product-categories.webp</x:v>
       </x:c>
       <x:c r="J26" s="56" t="str">
         <x:v>blog/vitaran-hp-professional-guide.html; blog/vitaran-i-professional-guide.html; blog/vitaran-s-professional-guide.html; blog/placentex-professional-guide.html; products.html</x:v>
@@ -3178,18 +3262,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L26" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M26" s="56"/>
-      <x:c r="N26" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M26" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/how-professional-buyers-compare-polynucleotide-product-categories.html</x:v>
+      </x:c>
+      <x:c r="N26" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O26" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P26" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q26" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -3235,10 +3323,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P27" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q27" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -3267,7 +3355,7 @@
         <x:v>profilo-structura-professional-guide</x:v>
       </x:c>
       <x:c r="I28" s="56" t="str">
-        <x:v>assets/products/profhilo-structura.webp</x:v>
+        <x:v>assets/products/profilo-structura-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J28" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/hybrid-hyaluronic-acid-vs-conventional-skin-boosters.html</x:v>
@@ -3276,18 +3364,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L28" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M28" s="56"/>
-      <x:c r="N28" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M28" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/profilo-structura-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N28" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O28" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P28" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q28" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -3316,7 +3408,7 @@
         <x:v>evehilo-professional-guide</x:v>
       </x:c>
       <x:c r="I29" s="56" t="str">
-        <x:v>assets/products/evehilo.webp</x:v>
+        <x:v>assets/products/evehilo-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J29" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/hybrid-hyaluronic-acid-vs-conventional-skin-boosters.html</x:v>
@@ -3325,18 +3417,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L29" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M29" s="56"/>
-      <x:c r="N29" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M29" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/evehilo-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N29" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O29" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P29" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q29" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -3365,7 +3461,7 @@
         <x:v>luhilo-professional-guide</x:v>
       </x:c>
       <x:c r="I30" s="56" t="str">
-        <x:v>assets/products/luhilo.webp</x:v>
+        <x:v>assets/products/luhilo-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J30" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/hybrid-hyaluronic-acid-vs-conventional-skin-boosters.html</x:v>
@@ -3374,18 +3470,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L30" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M30" s="56"/>
-      <x:c r="N30" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M30" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/luhilo-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N30" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O30" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P30" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q30" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -3414,7 +3514,7 @@
         <x:v>hybrid-hyaluronic-acid-vs-conventional-skin-boosters</x:v>
       </x:c>
       <x:c r="I31" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/hybrid-hyaluronic-acid-vs-conventional-skin-boosters.webp</x:v>
       </x:c>
       <x:c r="J31" s="56" t="str">
         <x:v>blog/profhilo-h-plusl-professional-guide.html; blog/profilo-structura-professional-guide.html; blog/evehilo-professional-guide.html; blog/luhilo-professional-guide.html; products.html</x:v>
@@ -3423,18 +3523,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L31" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M31" s="56"/>
-      <x:c r="N31" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M31" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/hybrid-hyaluronic-acid-vs-conventional-skin-boosters.html</x:v>
+      </x:c>
+      <x:c r="N31" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O31" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P31" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q31" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -3463,7 +3567,7 @@
         <x:v>jalupro-classic-professional-guide</x:v>
       </x:c>
       <x:c r="I32" s="56" t="str">
-        <x:v>assets/products/jalupro-classic.webp</x:v>
+        <x:v>assets/products/jalupro-classic-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J32" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/jalupro-product-range-and-amino-acid-skin-booster-categories.html</x:v>
@@ -3472,18 +3576,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L32" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M32" s="56"/>
-      <x:c r="N32" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M32" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/jalupro-classic-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N32" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O32" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P32" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q32" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -3512,7 +3620,7 @@
         <x:v>jalupro-super-hydro-professional-guide</x:v>
       </x:c>
       <x:c r="I33" s="56" t="str">
-        <x:v>assets/products/jalupro-super-hydro.webp</x:v>
+        <x:v>assets/products/jalupro-super-hydro-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J33" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/jalupro-product-range-and-amino-acid-skin-booster-categories.html</x:v>
@@ -3521,18 +3629,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L33" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M33" s="56"/>
-      <x:c r="N33" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M33" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/jalupro-super-hydro-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N33" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O33" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P33" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q33" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -3561,7 +3673,7 @@
         <x:v>jalupro-hmw-professional-guide</x:v>
       </x:c>
       <x:c r="I34" s="56" t="str">
-        <x:v>assets/products/jalupro-hmw.webp</x:v>
+        <x:v>assets/products/jalupro-hmw-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J34" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/jalupro-product-range-and-amino-acid-skin-booster-categories.html</x:v>
@@ -3570,18 +3682,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L34" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M34" s="56"/>
-      <x:c r="N34" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M34" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/jalupro-hmw-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N34" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O34" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P34" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q34" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -3610,7 +3726,7 @@
         <x:v>jalupro-young-eye-professional-guide</x:v>
       </x:c>
       <x:c r="I35" s="56" t="str">
-        <x:v>assets/products/jalupro-young-eye.png</x:v>
+        <x:v>assets/products/jalupro-young-eye-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J35" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/jalupro-product-range-and-amino-acid-skin-booster-categories.html</x:v>
@@ -3619,18 +3735,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L35" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M35" s="56"/>
-      <x:c r="N35" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M35" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/jalupro-young-eye-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N35" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O35" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P35" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q35" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -3659,7 +3779,7 @@
         <x:v>jalupro-product-range-and-amino-acid-skin-booster-categories</x:v>
       </x:c>
       <x:c r="I36" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/jalupro-product-range-and-amino-acid-skin-booster-categories.webp</x:v>
       </x:c>
       <x:c r="J36" s="56" t="str">
         <x:v>blog/jalupro-classic-professional-guide.html; blog/jalupro-super-hydro-professional-guide.html; blog/jalupro-hmw-professional-guide.html; blog/jalupro-young-eye-professional-guide.html; products.html</x:v>
@@ -3668,18 +3788,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L36" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M36" s="56"/>
-      <x:c r="N36" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M36" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/jalupro-product-range-and-amino-acid-skin-booster-categories.html</x:v>
+      </x:c>
+      <x:c r="N36" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O36" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P36" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q36" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -3708,7 +3832,7 @@
         <x:v>nctf-5-bottles-professional-guide</x:v>
       </x:c>
       <x:c r="I37" s="56" t="str">
-        <x:v>assets/products/nctf-5-bottles.webp</x:v>
+        <x:v>assets/products/nctf-5-bottles-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J37" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-evaluate-multi-ingredient-revitalisation-products.html</x:v>
@@ -3717,18 +3841,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L37" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M37" s="56"/>
-      <x:c r="N37" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M37" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/nctf-5-bottles-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N37" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O37" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P37" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q37" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -3757,7 +3885,7 @@
         <x:v>nctf-10-bottles-professional-guide</x:v>
       </x:c>
       <x:c r="I38" s="56" t="str">
-        <x:v>assets/products/nctf-10-bottles.webp</x:v>
+        <x:v>assets/products/nctf-10-bottles-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J38" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-evaluate-multi-ingredient-revitalisation-products.html</x:v>
@@ -3766,18 +3894,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L38" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M38" s="56"/>
-      <x:c r="N38" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M38" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/nctf-10-bottles-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N38" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O38" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P38" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q38" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -3806,7 +3938,7 @@
         <x:v>filorga-pink-glow-x2-professional-guide</x:v>
       </x:c>
       <x:c r="I39" s="56" t="str">
-        <x:v>assets/products/filorga-pink-glow-x2.webp</x:v>
+        <x:v>assets/products/filorga-pink-glow-x2-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J39" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-evaluate-multi-ingredient-revitalisation-products.html</x:v>
@@ -3815,18 +3947,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L39" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M39" s="56"/>
-      <x:c r="N39" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M39" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/filorga-pink-glow-x2-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N39" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O39" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P39" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q39" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -3855,7 +3991,7 @@
         <x:v>pink-glow-professional-guide</x:v>
       </x:c>
       <x:c r="I40" s="56" t="str">
-        <x:v>assets/products/pink-glow.webp</x:v>
+        <x:v>assets/products/pink-glow-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J40" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-evaluate-multi-ingredient-revitalisation-products.html</x:v>
@@ -3864,18 +4000,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L40" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M40" s="56"/>
-      <x:c r="N40" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M40" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/pink-glow-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N40" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O40" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P40" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q40" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -3904,7 +4044,7 @@
         <x:v>how-to-evaluate-multi-ingredient-revitalisation-products</x:v>
       </x:c>
       <x:c r="I41" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/how-to-evaluate-multi-ingredient-revitalisation-products.webp</x:v>
       </x:c>
       <x:c r="J41" s="56" t="str">
         <x:v>blog/nctf-5-bottles-professional-guide.html; blog/nctf-10-bottles-professional-guide.html; blog/filorga-pink-glow-x2-professional-guide.html; blog/pink-glow-professional-guide.html; products.html</x:v>
@@ -3913,18 +4053,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L41" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M41" s="56"/>
-      <x:c r="N41" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M41" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/how-to-evaluate-multi-ingredient-revitalisation-products.html</x:v>
+      </x:c>
+      <x:c r="N41" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O41" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P41" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q41" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -3953,7 +4097,7 @@
         <x:v>rrs-ha-eyes-professional-guide</x:v>
       </x:c>
       <x:c r="I42" s="56" t="str">
-        <x:v>assets/products/rrs-ha-eyes.webp</x:v>
+        <x:v>assets/products/rrs-ha-eyes-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J42" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/why-the-eye-area-requires-different-product-evaluation.html</x:v>
@@ -3962,18 +4106,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L42" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M42" s="56"/>
-      <x:c r="N42" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M42" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/rrs-ha-eyes-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N42" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O42" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P42" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q42" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -4002,7 +4150,7 @@
         <x:v>lumi-eyes-professional-guide</x:v>
       </x:c>
       <x:c r="I43" s="56" t="str">
-        <x:v>assets/products/lumi-eyes.webp</x:v>
+        <x:v>assets/products/lumi-eyes-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J43" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/why-the-eye-area-requires-different-product-evaluation.html</x:v>
@@ -4011,18 +4159,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L43" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M43" s="56"/>
-      <x:c r="N43" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M43" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/lumi-eyes-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N43" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O43" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P43" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q43" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -4051,7 +4203,7 @@
         <x:v>richese-eyes-professional-guide</x:v>
       </x:c>
       <x:c r="I44" s="56" t="str">
-        <x:v>assets/products/richese-eyes.webp</x:v>
+        <x:v>assets/products/richese-eyes-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J44" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/why-the-eye-area-requires-different-product-evaluation.html</x:v>
@@ -4060,18 +4212,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L44" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M44" s="56"/>
-      <x:c r="N44" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M44" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/richese-eyes-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N44" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O44" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P44" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q44" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -4100,7 +4256,7 @@
         <x:v>luna-eyes-professional-guide</x:v>
       </x:c>
       <x:c r="I45" s="56" t="str">
-        <x:v>assets/products/luna-eyes.webp</x:v>
+        <x:v>assets/products/luna-eyes-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J45" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/why-the-eye-area-requires-different-product-evaluation.html</x:v>
@@ -4109,18 +4265,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L45" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M45" s="56"/>
-      <x:c r="N45" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M45" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/luna-eyes-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N45" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O45" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P45" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q45" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -4149,7 +4309,7 @@
         <x:v>why-the-eye-area-requires-different-product-evaluation</x:v>
       </x:c>
       <x:c r="I46" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/why-the-eye-area-requires-different-product-evaluation.webp</x:v>
       </x:c>
       <x:c r="J46" s="56" t="str">
         <x:v>blog/rrs-ha-eyes-professional-guide.html; blog/lumi-eyes-professional-guide.html; blog/richese-eyes-professional-guide.html; blog/luna-eyes-professional-guide.html; products.html</x:v>
@@ -4158,18 +4318,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L46" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M46" s="56"/>
-      <x:c r="N46" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M46" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/why-the-eye-area-requires-different-product-evaluation.html</x:v>
+      </x:c>
+      <x:c r="N46" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O46" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P46" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q46" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -4215,10 +4379,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P47" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q47" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -4247,7 +4411,7 @@
         <x:v>exocode-professional-guide</x:v>
       </x:c>
       <x:c r="I48" s="56" t="str">
-        <x:v>assets/products/exocode.webp</x:v>
+        <x:v>assets/products/exocode-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J48" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/exosome-skin-boosters-evidence-terminology-and-sourcing-checks.html</x:v>
@@ -4256,18 +4420,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L48" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M48" s="56"/>
-      <x:c r="N48" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M48" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/exocode-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N48" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O48" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P48" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q48" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -4296,7 +4464,7 @@
         <x:v>exoten-professional-guide</x:v>
       </x:c>
       <x:c r="I49" s="56" t="str">
-        <x:v>assets/products/exoten.webp</x:v>
+        <x:v>assets/products/exoten-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J49" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/exosome-skin-boosters-evidence-terminology-and-sourcing-checks.html</x:v>
@@ -4305,18 +4473,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L49" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M49" s="56"/>
-      <x:c r="N49" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M49" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/exoten-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N49" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O49" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P49" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q49" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -4345,7 +4517,7 @@
         <x:v>p-cell-professional-guide</x:v>
       </x:c>
       <x:c r="I50" s="56" t="str">
-        <x:v>assets/products/p-cell.webp</x:v>
+        <x:v>assets/products/p-cell-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J50" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/exosome-skin-boosters-evidence-terminology-and-sourcing-checks.html</x:v>
@@ -4354,18 +4526,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L50" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M50" s="56"/>
-      <x:c r="N50" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M50" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/p-cell-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N50" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O50" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P50" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q50" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -4394,7 +4570,7 @@
         <x:v>exosome-skin-boosters-evidence-terminology-and-sourcing-checks</x:v>
       </x:c>
       <x:c r="I51" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/exosome-skin-boosters-evidence-terminology-and-sourcing-checks.webp</x:v>
       </x:c>
       <x:c r="J51" s="56" t="str">
         <x:v>blog/complex-asce-professional-guide.html; blog/exocode-professional-guide.html; blog/exoten-professional-guide.html; blog/p-cell-professional-guide.html; products.html</x:v>
@@ -4403,18 +4579,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L51" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M51" s="56"/>
-      <x:c r="N51" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M51" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/exosome-skin-boosters-evidence-terminology-and-sourcing-checks.html</x:v>
+      </x:c>
+      <x:c r="N51" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O51" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P51" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q51" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -4443,7 +4623,7 @@
         <x:v>karisma-professional-guide</x:v>
       </x:c>
       <x:c r="I52" s="56" t="str">
-        <x:v>assets/products/karisma.webp</x:v>
+        <x:v>assets/products/karisma-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J52" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/collagen-biostimulator-categories-compared-for-professional-buyers.html</x:v>
@@ -4452,18 +4632,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L52" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M52" s="56"/>
-      <x:c r="N52" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M52" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/karisma-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N52" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O52" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P52" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q52" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -4509,10 +4693,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P53" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q53" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -4558,10 +4742,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P54" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q54" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -4607,10 +4791,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P55" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q55" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -4639,7 +4823,7 @@
         <x:v>collagen-biostimulator-categories-compared-for-professional-buyers</x:v>
       </x:c>
       <x:c r="I56" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/collagen-biostimulator-categories-compared-for-professional-buyers.webp</x:v>
       </x:c>
       <x:c r="J56" s="56" t="str">
         <x:v>blog/karisma-professional-guide.html; blog/juvelook-professional-guide.html; blog/gouri-professional-guide.html; blog/olidia-plla-professional-guide.html; products.html</x:v>
@@ -4648,18 +4832,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L56" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M56" s="56"/>
-      <x:c r="N56" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M56" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/collagen-biostimulator-categories-compared-for-professional-buyers.html</x:v>
+      </x:c>
+      <x:c r="N56" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O56" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P56" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q56" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -4705,10 +4893,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P57" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q57" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -4754,10 +4942,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P58" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q58" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -4803,10 +4991,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P59" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q59" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -4852,10 +5040,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P60" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q60" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -4884,7 +5072,7 @@
         <x:v>how-to-compare-korean-dermal-filler-brands-and-product-families</x:v>
       </x:c>
       <x:c r="I61" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/how-to-compare-korean-dermal-filler-brands-and-product-families.webp</x:v>
       </x:c>
       <x:c r="J61" s="56" t="str">
         <x:v>blog/neuramis-professional-guide.html; blog/revolax-professional-guide.html; blog/dermalax-professional-guide.html; blog/chaeum-professional-guide.html; products.html</x:v>
@@ -4893,18 +5081,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L61" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M61" s="56"/>
-      <x:c r="N61" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M61" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/how-to-compare-korean-dermal-filler-brands-and-product-families.html</x:v>
+      </x:c>
+      <x:c r="N61" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O61" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P61" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q61" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -4950,10 +5142,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P62" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q62" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -4999,10 +5191,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P63" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q63" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -5048,10 +5240,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P64" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q64" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -5097,10 +5289,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P65" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q65" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -5129,7 +5321,7 @@
         <x:v>how-to-evaluate-dermal-filler-product-families-by-intended-category</x:v>
       </x:c>
       <x:c r="I66" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/how-to-evaluate-dermal-filler-product-families-by-intended-category.webp</x:v>
       </x:c>
       <x:c r="J66" s="56" t="str">
         <x:v>blog/juvederm-voluma-professional-guide.html; blog/restylane-defyne-professional-guide.html; blog/restylane-refyne-professional-guide.html; blog/stylage-vivacy-professional-guide.html; products.html</x:v>
@@ -5138,18 +5330,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L66" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M66" s="56"/>
-      <x:c r="N66" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M66" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/how-to-evaluate-dermal-filler-product-families-by-intended-category.html</x:v>
+      </x:c>
+      <x:c r="N66" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O66" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P66" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q66" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -5195,10 +5391,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P67" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q67" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -5244,10 +5440,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P68" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q68" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -5293,10 +5489,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P69" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q69" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -5342,10 +5538,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P70" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q70" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -5374,7 +5570,7 @@
         <x:v>lip-filler-product-comparison-questions-professional-buyers-should-ask</x:v>
       </x:c>
       <x:c r="I71" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/lip-filler-product-comparison-questions-professional-buyers-should-ask.webp</x:v>
       </x:c>
       <x:c r="J71" s="56" t="str">
         <x:v>blog/restylane-kysse-professional-guide.html; blog/juvederm-vobela-professional-guide.html; blog/eptq-professional-guide.html; blog/elasty-professional-guide.html; products.html</x:v>
@@ -5383,18 +5579,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L71" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M71" s="56"/>
-      <x:c r="N71" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M71" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/lip-filler-product-comparison-questions-professional-buyers-should-ask.html</x:v>
+      </x:c>
+      <x:c r="N71" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O71" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P71" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q71" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -5440,10 +5640,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P72" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q72" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -5489,10 +5689,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P73" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q73" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -5538,10 +5738,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P74" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q74" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -5587,10 +5787,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P75" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q75" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -5619,7 +5819,7 @@
         <x:v>body-filler-sourcing-safety-documentation-and-local-regulation-checks</x:v>
       </x:c>
       <x:c r="I76" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/body-filler-sourcing-safety-documentation-and-local-regulation-checks.webp</x:v>
       </x:c>
       <x:c r="J76" s="56" t="str">
         <x:v>blog/jariot-body-professional-guide.html; blog/helios-body-professional-guide.html; blog/maxxyfill-body-professional-guide.html; blog/sedy-fill-body-professional-guide.html; products.html</x:v>
@@ -5628,18 +5828,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L76" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M76" s="56"/>
-      <x:c r="N76" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M76" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/body-filler-sourcing-safety-documentation-and-local-regulation-checks.html</x:v>
+      </x:c>
+      <x:c r="N76" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O76" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P76" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q76" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -5685,10 +5889,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P77" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q77" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -5734,10 +5938,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P78" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q78" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -5783,10 +5987,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P79" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q79" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -5832,10 +6036,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P80" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q80" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -5864,7 +6068,7 @@
         <x:v>how-botulinum-toxin-product-families-differ-for-professional-procurement</x:v>
       </x:c>
       <x:c r="I81" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/how-botulinum-toxin-product-families-differ-for-professional-procurement.webp</x:v>
       </x:c>
       <x:c r="J81" s="56" t="str">
         <x:v>blog/nabota-100-professional-guide.html; blog/botulax-100-professional-guide.html; blog/innotox-50-professional-guide.html; blog/xeomin-professional-guide.html; products.html</x:v>
@@ -5873,18 +6077,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L81" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M81" s="56"/>
-      <x:c r="N81" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M81" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/how-botulinum-toxin-product-families-differ-for-professional-procurement.html</x:v>
+      </x:c>
+      <x:c r="N81" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O81" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P81" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q81" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -5930,10 +6138,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P82" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q82" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -5979,10 +6187,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P83" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q83" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -6028,10 +6236,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P84" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q84" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -6077,10 +6285,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P85" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q85" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -6109,7 +6317,7 @@
         <x:v>cold-chain-and-documentation-checks-for-korean-botulinum-toxin-products</x:v>
       </x:c>
       <x:c r="I86" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/cold-chain-and-documentation-checks-for-korean-botulinum-toxin-products.webp</x:v>
       </x:c>
       <x:c r="J86" s="56" t="str">
         <x:v>blog/wondertox-100-professional-guide.html; blog/hutox-100-professional-guide.html; blog/coretox-100-professional-guide.html; blog/toxta-100-professional-guide.html; products.html</x:v>
@@ -6118,18 +6326,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L86" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M86" s="56"/>
-      <x:c r="N86" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M86" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/cold-chain-and-documentation-checks-for-korean-botulinum-toxin-products.html</x:v>
+      </x:c>
+      <x:c r="N86" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O86" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P86" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q86" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -6175,10 +6387,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P87" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q87" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -6224,10 +6436,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P88" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q88" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -6273,10 +6485,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P89" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q89" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -6322,10 +6534,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P90" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q90" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -6354,7 +6566,7 @@
         <x:v>body-contouring-products-evidence-claims-and-buyer-due-diligence</x:v>
       </x:c>
       <x:c r="I91" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/body-contouring-products-evidence-claims-and-buyer-due-diligence.webp</x:v>
       </x:c>
       <x:c r="J91" s="56" t="str">
         <x:v>blog/aqualyx-professional-guide.html; blog/lipolab-professional-guide.html; blog/lemon-bottle-professional-guide.html; blog/kabelline-professional-guide.html; products.html</x:v>
@@ -6363,18 +6575,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L91" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M91" s="56"/>
-      <x:c r="N91" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M91" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/body-contouring-products-evidence-claims-and-buyer-due-diligence.html</x:v>
+      </x:c>
+      <x:c r="N91" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O91" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P91" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q91" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -6420,10 +6636,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P92" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q92" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -6469,10 +6685,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P93" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q93" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -6518,10 +6734,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P94" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q94" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -6567,10 +6783,10 @@
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P95" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q95" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -6599,7 +6815,7 @@
         <x:v>topical-anaesthetic-products-concentration-labelling-and-local-regulations</x:v>
       </x:c>
       <x:c r="I96" s="56" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/topical-anaesthetic-products-concentration-labelling-and-local-regulations.webp</x:v>
       </x:c>
       <x:c r="J96" s="56" t="str">
         <x:v>blog/korean-medicaine-professional-guide.html; blog/j-cain-10-56-professional-guide.html; blog/m-caine-cream-professional-guide.html; blog/lidocaine-cream-professional-guide.html; products.html</x:v>
@@ -6608,18 +6824,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L96" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M96" s="56"/>
-      <x:c r="N96" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M96" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/topical-anaesthetic-products-concentration-labelling-and-local-regulations.html</x:v>
+      </x:c>
+      <x:c r="N96" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O96" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P96" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q96" s="57" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -6648,7 +6868,7 @@
         <x:v>nucleofill-strong-professional-guide</x:v>
       </x:c>
       <x:c r="I97" s="56" t="str">
-        <x:v>assets/products/nucleofill-strong.webp</x:v>
+        <x:v>assets/products/nucleofill-strong-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J97" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-verify-aesthetic-product-authenticity-storage-and-shipping-records.html</x:v>
@@ -6657,18 +6877,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L97" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M97" s="56"/>
-      <x:c r="N97" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M97" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/nucleofill-strong-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N97" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O97" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P97" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q97" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -6697,7 +6921,7 @@
         <x:v>curenex-professional-guide</x:v>
       </x:c>
       <x:c r="I98" s="56" t="str">
-        <x:v>assets/products/curenex.webp</x:v>
+        <x:v>assets/products/curenex-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J98" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-verify-aesthetic-product-authenticity-storage-and-shipping-records.html</x:v>
@@ -6706,18 +6930,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L98" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M98" s="56"/>
-      <x:c r="N98" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M98" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/curenex-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N98" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O98" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P98" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q98" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -6746,7 +6974,7 @@
         <x:v>revok-50-professional-guide</x:v>
       </x:c>
       <x:c r="I99" s="56" t="str">
-        <x:v>assets/products/revok-50.webp</x:v>
+        <x:v>assets/products/revok-50-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J99" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-verify-aesthetic-product-authenticity-storage-and-shipping-records.html</x:v>
@@ -6755,18 +6983,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L99" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M99" s="56"/>
-      <x:c r="N99" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M99" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/revok-50-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N99" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O99" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P99" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q99" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -6795,7 +7027,7 @@
         <x:v>teoxan-1-professional-guide</x:v>
       </x:c>
       <x:c r="I100" s="56" t="str">
-        <x:v>assets/products/teoxan-1.webp</x:v>
+        <x:v>assets/products/teoxan-1-professional-guide.webp</x:v>
       </x:c>
       <x:c r="J100" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-verify-aesthetic-product-authenticity-storage-and-shipping-records.html</x:v>
@@ -6804,18 +7036,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L100" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M100" s="56"/>
-      <x:c r="N100" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M100" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/teoxan-1-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N100" s="49" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O100" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P100" s="49" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q100" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -6844,7 +7080,7 @@
         <x:v>how-to-verify-aesthetic-product-authenticity-storage-and-shipping-records</x:v>
       </x:c>
       <x:c r="I101" s="59" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/how-to-verify-aesthetic-product-authenticity-storage-and-shipping-records.webp</x:v>
       </x:c>
       <x:c r="J101" s="59" t="str">
         <x:v>blog/nucleofill-strong-professional-guide.html; blog/curenex-professional-guide.html; blog/revok-50-professional-guide.html; blog/teoxan-1-professional-guide.html; products.html</x:v>
@@ -6853,18 +7089,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L101" s="59" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M101" s="59"/>
-      <x:c r="N101" s="50"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M101" s="59" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/how-to-verify-aesthetic-product-authenticity-storage-and-shipping-records.html</x:v>
+      </x:c>
+      <x:c r="N101" s="50" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O101" s="59" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P101" s="50" t="n">
-        <x:v>46295</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q101" s="60" t="str">
-        <x:v>Pillar article for the preceding four product articles. Educational value first; subtle commercial CTA. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -6893,7 +7133,7 @@
         <x:v>skin-booster-vs-serum-hydration-texture-and-glow</x:v>
       </x:c>
       <x:c r="I102" s="61" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/skin-booster-vs-serum-hydration-texture-and-glow.webp</x:v>
       </x:c>
       <x:c r="J102" s="61" t="str">
         <x:v>blog/vs-pnad-plus-professional-guide.html; blog/vs-vitathione-nad-plus-skin-glow-guide.html; blog/skinfill-bacio-wholesale-sourcing.html; products.html</x:v>
@@ -6902,18 +7142,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L102" s="61" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M102" s="61"/>
-      <x:c r="N102" s="62"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M102" s="61" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/skin-booster-vs-serum-hydration-texture-and-glow.html</x:v>
+      </x:c>
+      <x:c r="N102" s="62" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O102" s="61" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P102" s="62" t="n">
-        <x:v>46298</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q102" s="61" t="str">
-        <x:v>Distinct content-gap article comparing daily topical care with professional product categories. Educational value first; no procedure instructions. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -6942,7 +7186,7 @@
         <x:v>sensitive-skin-checklist-professional-aesthetic-products</x:v>
       </x:c>
       <x:c r="I103" s="61" t="str">
-        <x:v>GENERATE_BRANDED_EDUCATIONAL_IMAGE</x:v>
+        <x:v>assets/blog/sensitive-skin-checklist-professional-aesthetic-products.webp</x:v>
       </x:c>
       <x:c r="J103" s="61" t="str">
         <x:v>blog/korean-aesthetic-product-supplier.html; blog/puri-lips-wholesale-sourcing.html; blog/vs-pnad-plus-professional-guide.html; products.html; contact.html</x:v>
@@ -6951,18 +7195,22 @@
         <x:v>Use PubMed, NIH, FDA/WHO or professional guidance where relevant; verify every URL before publication</x:v>
       </x:c>
       <x:c r="L103" s="61" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M103" s="61"/>
-      <x:c r="N103" s="62"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M103" s="61" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/sensitive-skin-checklist-professional-aesthetic-products.html</x:v>
+      </x:c>
+      <x:c r="N103" s="62" t="n">
+        <x:v>46299</x:v>
+      </x:c>
       <x:c r="O103" s="61" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P103" s="62" t="n">
-        <x:v>46298</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="Q103" s="61" t="str">
-        <x:v>Distinct content-gap article for readers with reactive or barrier-stressed skin. Avoid diagnosis and recommend qualified consultation. Batch publishing is paused until the user confirms that the full campaign is ready to publish together.</x:v>
+        <x:v>Published in the verified 2026-10-04 batch. Live article and image returned HTTP 200; daily automation remains paused.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6985,7 +7233,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re195fc59678a4741"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4518d23df0d54a6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7637,7 +7885,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79ad121cef434411"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5834f7400494ad3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7853,7 +8101,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0136d7777f0b4e83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b305563ee694c1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete 100-article SEO campaign tracking
</commit_message>
<xml_diff>
--- a/seo-automation/sowena-seo-master-tracker.xlsx
+++ b/seo-automation/sowena-seo-master-tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R699c1091a7bf4415"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="2" r:id="Ra25c7075a89c4c66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap 100" sheetId="3" r:id="Ra81c42edcfe54bec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Links" sheetId="4" r:id="R1eb16988072b45b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Notes" sheetId="5" r:id="Raa454c8245364d4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rae87130e77ec4bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="2" r:id="Rda5cd8f958c9474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap 100" sheetId="3" r:id="Re533cd20ceeb4f85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Links" sheetId="4" r:id="R6606e4e9ca27402b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and Notes" sheetId="5" r:id="Raf4bc91f79364190"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -984,7 +984,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="20" t="str">
-        <x:v>Campaign status: 63 of 100 additional articles are live. The remaining 37 product articles are on hold until approved product images are added. Daily publishing automation remains paused.</x:v>
+        <x:v>Campaign complete: all 100 additional articles are live. The final 37 use disclosed GPT-designed category editorial covers that can be replaced with approved clean product photographs later. Daily publishing automation remains paused.</x:v>
       </x:c>
     </x:row>
     <x:row r="14"/>
@@ -1840,7 +1840,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4711cb6e0fe6450d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95eed674c388488c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3306,7 +3306,7 @@
         <x:v>profhilo-h-plusl-professional-guide</x:v>
       </x:c>
       <x:c r="I27" s="56" t="str">
-        <x:v>assets/products/profhilo-h-l.webp</x:v>
+        <x:v>assets/blog/gpt-category-covers/hybrid-ha-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J27" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/hybrid-hyaluronic-acid-vs-conventional-skin-boosters.html</x:v>
@@ -3315,18 +3315,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L27" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M27" s="56"/>
-      <x:c r="N27" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M27" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/profhilo-h-plusl-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N27" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O27" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P27" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q27" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -4362,7 +4366,7 @@
         <x:v>complex-asce-professional-guide</x:v>
       </x:c>
       <x:c r="I47" s="56" t="str">
-        <x:v>assets/products/complex-asce.webp</x:v>
+        <x:v>assets/blog/gpt-category-covers/exosome-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J47" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/exosome-skin-boosters-evidence-terminology-and-sourcing-checks.html</x:v>
@@ -4371,18 +4375,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L47" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M47" s="56"/>
-      <x:c r="N47" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M47" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/complex-asce-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N47" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O47" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P47" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q47" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -4676,7 +4684,7 @@
         <x:v>juvelook-professional-guide</x:v>
       </x:c>
       <x:c r="I53" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/collagen-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J53" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/collagen-biostimulator-categories-compared-for-professional-buyers.html</x:v>
@@ -4685,18 +4693,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L53" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M53" s="56"/>
-      <x:c r="N53" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M53" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/juvelook-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N53" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O53" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P53" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q53" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -4725,7 +4737,7 @@
         <x:v>gouri-professional-guide</x:v>
       </x:c>
       <x:c r="I54" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/collagen-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J54" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/collagen-biostimulator-categories-compared-for-professional-buyers.html</x:v>
@@ -4734,18 +4746,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L54" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M54" s="56"/>
-      <x:c r="N54" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M54" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/gouri-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N54" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O54" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P54" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q54" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -4774,7 +4790,7 @@
         <x:v>olidia-plla-professional-guide</x:v>
       </x:c>
       <x:c r="I55" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/collagen-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J55" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/collagen-biostimulator-categories-compared-for-professional-buyers.html</x:v>
@@ -4783,18 +4799,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L55" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M55" s="56"/>
-      <x:c r="N55" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M55" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/olidia-plla-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N55" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O55" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P55" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q55" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -4876,7 +4896,7 @@
         <x:v>neuramis-professional-guide</x:v>
       </x:c>
       <x:c r="I57" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J57" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-compare-korean-dermal-filler-brands-and-product-families.html</x:v>
@@ -4885,18 +4905,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L57" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M57" s="56"/>
-      <x:c r="N57" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M57" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/neuramis-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N57" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O57" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P57" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q57" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -4925,7 +4949,7 @@
         <x:v>revolax-professional-guide</x:v>
       </x:c>
       <x:c r="I58" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J58" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-compare-korean-dermal-filler-brands-and-product-families.html</x:v>
@@ -4934,18 +4958,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L58" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M58" s="56"/>
-      <x:c r="N58" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M58" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/revolax-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N58" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O58" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P58" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q58" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -4974,7 +5002,7 @@
         <x:v>dermalax-professional-guide</x:v>
       </x:c>
       <x:c r="I59" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J59" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-compare-korean-dermal-filler-brands-and-product-families.html</x:v>
@@ -4983,18 +5011,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L59" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M59" s="56"/>
-      <x:c r="N59" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M59" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/dermalax-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N59" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O59" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P59" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q59" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -5023,7 +5055,7 @@
         <x:v>chaeum-professional-guide</x:v>
       </x:c>
       <x:c r="I60" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J60" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-compare-korean-dermal-filler-brands-and-product-families.html</x:v>
@@ -5032,18 +5064,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L60" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M60" s="56"/>
-      <x:c r="N60" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M60" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/chaeum-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N60" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O60" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P60" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q60" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -5125,7 +5161,7 @@
         <x:v>juvederm-voluma-professional-guide</x:v>
       </x:c>
       <x:c r="I62" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J62" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-evaluate-dermal-filler-product-families-by-intended-category.html</x:v>
@@ -5134,18 +5170,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L62" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M62" s="56"/>
-      <x:c r="N62" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M62" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/juvederm-voluma-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N62" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O62" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P62" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q62" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -5174,7 +5214,7 @@
         <x:v>restylane-defyne-professional-guide</x:v>
       </x:c>
       <x:c r="I63" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J63" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-evaluate-dermal-filler-product-families-by-intended-category.html</x:v>
@@ -5183,18 +5223,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L63" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M63" s="56"/>
-      <x:c r="N63" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M63" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/restylane-defyne-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N63" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O63" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P63" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q63" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -5223,7 +5267,7 @@
         <x:v>restylane-refyne-professional-guide</x:v>
       </x:c>
       <x:c r="I64" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J64" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-evaluate-dermal-filler-product-families-by-intended-category.html</x:v>
@@ -5232,18 +5276,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L64" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M64" s="56"/>
-      <x:c r="N64" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M64" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/restylane-refyne-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N64" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O64" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P64" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q64" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -5272,7 +5320,7 @@
         <x:v>stylage-vivacy-professional-guide</x:v>
       </x:c>
       <x:c r="I65" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J65" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-to-evaluate-dermal-filler-product-families-by-intended-category.html</x:v>
@@ -5281,18 +5329,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L65" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M65" s="56"/>
-      <x:c r="N65" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M65" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/stylage-vivacy-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N65" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O65" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P65" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q65" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -5374,7 +5426,7 @@
         <x:v>restylane-kysse-professional-guide</x:v>
       </x:c>
       <x:c r="I67" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J67" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/lip-filler-product-comparison-questions-professional-buyers-should-ask.html</x:v>
@@ -5383,18 +5435,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L67" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M67" s="56"/>
-      <x:c r="N67" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M67" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/restylane-kysse-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N67" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O67" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P67" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q67" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -5423,7 +5479,7 @@
         <x:v>juvederm-vobela-professional-guide</x:v>
       </x:c>
       <x:c r="I68" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J68" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/lip-filler-product-comparison-questions-professional-buyers-should-ask.html</x:v>
@@ -5432,18 +5488,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L68" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M68" s="56"/>
-      <x:c r="N68" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M68" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/juvederm-vobela-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N68" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O68" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P68" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q68" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -5472,7 +5532,7 @@
         <x:v>eptq-professional-guide</x:v>
       </x:c>
       <x:c r="I69" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J69" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/lip-filler-product-comparison-questions-professional-buyers-should-ask.html</x:v>
@@ -5481,18 +5541,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L69" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M69" s="56"/>
-      <x:c r="N69" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M69" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/eptq-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N69" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O69" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P69" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q69" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -5521,7 +5585,7 @@
         <x:v>elasty-professional-guide</x:v>
       </x:c>
       <x:c r="I70" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/facial-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J70" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/lip-filler-product-comparison-questions-professional-buyers-should-ask.html</x:v>
@@ -5530,18 +5594,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L70" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M70" s="56"/>
-      <x:c r="N70" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M70" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/elasty-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N70" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O70" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P70" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q70" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -5623,7 +5691,7 @@
         <x:v>jariot-body-professional-guide</x:v>
       </x:c>
       <x:c r="I72" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/body-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J72" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/body-filler-sourcing-safety-documentation-and-local-regulation-checks.html</x:v>
@@ -5632,18 +5700,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L72" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M72" s="56"/>
-      <x:c r="N72" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M72" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/jariot-body-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N72" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O72" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P72" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q72" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -5672,7 +5744,7 @@
         <x:v>helios-body-professional-guide</x:v>
       </x:c>
       <x:c r="I73" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/body-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J73" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/body-filler-sourcing-safety-documentation-and-local-regulation-checks.html</x:v>
@@ -5681,18 +5753,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L73" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M73" s="56"/>
-      <x:c r="N73" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M73" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/helios-body-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N73" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O73" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P73" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q73" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -5721,7 +5797,7 @@
         <x:v>maxxyfill-body-professional-guide</x:v>
       </x:c>
       <x:c r="I74" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/body-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J74" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/body-filler-sourcing-safety-documentation-and-local-regulation-checks.html</x:v>
@@ -5730,18 +5806,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L74" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M74" s="56"/>
-      <x:c r="N74" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M74" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/maxxyfill-body-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N74" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O74" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P74" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q74" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -5770,7 +5850,7 @@
         <x:v>sedy-fill-body-professional-guide</x:v>
       </x:c>
       <x:c r="I75" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/body-filler-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J75" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/body-filler-sourcing-safety-documentation-and-local-regulation-checks.html</x:v>
@@ -5779,18 +5859,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L75" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M75" s="56"/>
-      <x:c r="N75" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M75" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/sedy-fill-body-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N75" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O75" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P75" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q75" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -5872,7 +5956,7 @@
         <x:v>nabota-100-professional-guide</x:v>
       </x:c>
       <x:c r="I77" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/botulinum-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J77" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-botulinum-toxin-product-families-differ-for-professional-procurement.html</x:v>
@@ -5881,18 +5965,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L77" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M77" s="56"/>
-      <x:c r="N77" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M77" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/nabota-100-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N77" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O77" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P77" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q77" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -5921,7 +6009,7 @@
         <x:v>botulax-100-professional-guide</x:v>
       </x:c>
       <x:c r="I78" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/botulinum-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J78" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-botulinum-toxin-product-families-differ-for-professional-procurement.html</x:v>
@@ -5930,18 +6018,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L78" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M78" s="56"/>
-      <x:c r="N78" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M78" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/botulax-100-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N78" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O78" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P78" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q78" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -5970,7 +6062,7 @@
         <x:v>innotox-50-professional-guide</x:v>
       </x:c>
       <x:c r="I79" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/botulinum-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J79" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-botulinum-toxin-product-families-differ-for-professional-procurement.html</x:v>
@@ -5979,18 +6071,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L79" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M79" s="56"/>
-      <x:c r="N79" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M79" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/innotox-50-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N79" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O79" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P79" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q79" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -6019,7 +6115,7 @@
         <x:v>xeomin-professional-guide</x:v>
       </x:c>
       <x:c r="I80" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/botulinum-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J80" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/how-botulinum-toxin-product-families-differ-for-professional-procurement.html</x:v>
@@ -6028,18 +6124,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L80" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M80" s="56"/>
-      <x:c r="N80" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M80" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/xeomin-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N80" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O80" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P80" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q80" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -6121,7 +6221,7 @@
         <x:v>wondertox-100-professional-guide</x:v>
       </x:c>
       <x:c r="I82" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/botulinum-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J82" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/cold-chain-and-documentation-checks-for-korean-botulinum-toxin-products.html</x:v>
@@ -6130,18 +6230,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L82" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M82" s="56"/>
-      <x:c r="N82" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M82" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/wondertox-100-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N82" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O82" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P82" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q82" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -6170,7 +6274,7 @@
         <x:v>hutox-100-professional-guide</x:v>
       </x:c>
       <x:c r="I83" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/botulinum-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J83" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/cold-chain-and-documentation-checks-for-korean-botulinum-toxin-products.html</x:v>
@@ -6179,18 +6283,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L83" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M83" s="56"/>
-      <x:c r="N83" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M83" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/hutox-100-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N83" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O83" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P83" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q83" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -6219,7 +6327,7 @@
         <x:v>coretox-100-professional-guide</x:v>
       </x:c>
       <x:c r="I84" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/botulinum-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J84" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/cold-chain-and-documentation-checks-for-korean-botulinum-toxin-products.html</x:v>
@@ -6228,18 +6336,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L84" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M84" s="56"/>
-      <x:c r="N84" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M84" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/coretox-100-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N84" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O84" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P84" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q84" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -6268,7 +6380,7 @@
         <x:v>toxta-100-professional-guide</x:v>
       </x:c>
       <x:c r="I85" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/botulinum-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J85" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/cold-chain-and-documentation-checks-for-korean-botulinum-toxin-products.html</x:v>
@@ -6277,18 +6389,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L85" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M85" s="56"/>
-      <x:c r="N85" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M85" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/toxta-100-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N85" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O85" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P85" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q85" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -6370,7 +6486,7 @@
         <x:v>aqualyx-professional-guide</x:v>
       </x:c>
       <x:c r="I87" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/body-contouring-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J87" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/body-contouring-products-evidence-claims-and-buyer-due-diligence.html</x:v>
@@ -6379,18 +6495,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L87" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M87" s="56"/>
-      <x:c r="N87" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M87" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/aqualyx-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N87" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O87" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P87" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q87" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -6419,7 +6539,7 @@
         <x:v>lipolab-professional-guide</x:v>
       </x:c>
       <x:c r="I88" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/body-contouring-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J88" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/body-contouring-products-evidence-claims-and-buyer-due-diligence.html</x:v>
@@ -6428,18 +6548,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L88" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M88" s="56"/>
-      <x:c r="N88" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M88" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/lipolab-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N88" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O88" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P88" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q88" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -6468,7 +6592,7 @@
         <x:v>lemon-bottle-professional-guide</x:v>
       </x:c>
       <x:c r="I89" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/body-contouring-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J89" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/body-contouring-products-evidence-claims-and-buyer-due-diligence.html</x:v>
@@ -6477,18 +6601,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L89" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M89" s="56"/>
-      <x:c r="N89" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M89" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/lemon-bottle-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N89" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O89" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P89" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q89" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -6517,7 +6645,7 @@
         <x:v>kabelline-professional-guide</x:v>
       </x:c>
       <x:c r="I90" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/body-contouring-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J90" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/body-contouring-products-evidence-claims-and-buyer-due-diligence.html</x:v>
@@ -6526,18 +6654,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L90" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M90" s="56"/>
-      <x:c r="N90" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M90" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/kabelline-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N90" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O90" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P90" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q90" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -6619,7 +6751,7 @@
         <x:v>korean-medicaine-professional-guide</x:v>
       </x:c>
       <x:c r="I92" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/topical-anaesthetic-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J92" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/topical-anaesthetic-products-concentration-labelling-and-local-regulations.html</x:v>
@@ -6628,18 +6760,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L92" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M92" s="56"/>
-      <x:c r="N92" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M92" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/korean-medicaine-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N92" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O92" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P92" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q92" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -6668,7 +6804,7 @@
         <x:v>j-cain-10-56-professional-guide</x:v>
       </x:c>
       <x:c r="I93" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/topical-anaesthetic-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J93" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/topical-anaesthetic-products-concentration-labelling-and-local-regulations.html</x:v>
@@ -6677,18 +6813,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L93" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M93" s="56"/>
-      <x:c r="N93" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M93" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/j-cain-10-56-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N93" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O93" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P93" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q93" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -6717,7 +6857,7 @@
         <x:v>m-caine-cream-professional-guide</x:v>
       </x:c>
       <x:c r="I94" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/topical-anaesthetic-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J94" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/topical-anaesthetic-products-concentration-labelling-and-local-regulations.html</x:v>
@@ -6726,18 +6866,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L94" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M94" s="56"/>
-      <x:c r="N94" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M94" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/m-caine-cream-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N94" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O94" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P94" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q94" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -6766,7 +6910,7 @@
         <x:v>lidocaine-cream-professional-guide</x:v>
       </x:c>
       <x:c r="I95" s="56" t="str">
-        <x:v>VERIFY_APPROVED_SOURCE_FOLDER</x:v>
+        <x:v>assets/blog/gpt-category-covers/topical-anaesthetic-gpt-editorial.webp</x:v>
       </x:c>
       <x:c r="J95" s="56" t="str">
         <x:v>products.html; contact.html; planned pillar: blog/topical-anaesthetic-products-concentration-labelling-and-local-regulations.html</x:v>
@@ -6775,18 +6919,22 @@
         <x:v>Verify official manufacturer page; add 1-3 authoritative sources during research</x:v>
       </x:c>
       <x:c r="L95" s="56" t="str">
-        <x:v>BATCH HOLD</x:v>
-      </x:c>
-      <x:c r="M95" s="56"/>
-      <x:c r="N95" s="49"/>
+        <x:v>PUBLISHED</x:v>
+      </x:c>
+      <x:c r="M95" s="56" t="str">
+        <x:v>https://www.sowenabeauty.com/blog/lidocaine-cream-professional-guide.html</x:v>
+      </x:c>
+      <x:c r="N95" s="49" t="n">
+        <x:v>46301</x:v>
+      </x:c>
       <x:c r="O95" s="56" t="str">
         <x:v>NOT CHECKED</x:v>
       </x:c>
       <x:c r="P95" s="49" t="n">
-        <x:v>46299</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="Q95" s="57" t="str">
-        <x:v>Reader-first product education. Verify packaging, ingredients, manufacturer, evidence and local professional-use context before writing. Do not center wholesale or MOQ. Needs approved product background image. Needs approved product background image before publication; publish after the image is added.</x:v>
+        <x:v>Published live with a disclosed GPT-designed category editorial cover. The image is not product packaging; replace it when an approved clean product photograph is supplied. Live article and image returned HTTP 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -7233,7 +7381,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4518d23df0d54a6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6848df0d8d3648d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7885,7 +8033,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5834f7400494ad3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R550e717ada3841be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8101,7 +8249,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b305563ee694c1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43e66c380bdc432f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>